<commit_message>
fix(s1): no per-act debt to transfer while the 08 register is blocked
With the same advance entered both as «Оплата» and «Зачёт аванса» the
register total was blocked, but sheet «Долг по актам» still showed
500 000 / 300 000 in the columns the buyer copies into file 14. Now H and
J show «ЗАБЛОКИРОВАН», the row check names the blocked register and the act
is not marked for transfer. LibreOffice scenario C asserts it.

docProps/app.xml is pinned to the value already on main, so 04-ks-2-ks-3
is byte-identical to main again (its only diff was the openpyxl version).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ANyqChjMoEQrjdkzBWFdgh
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/08-uchet-obemov-peredachi-raschetov.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/08-uchet-obemov-peredachi-raschetov.xlsx
@@ -30693,7 +30693,7 @@
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>IF(OR(B5="",E5=""),"",F5-G5)</f>
+        <f>IF(OR(B5="",E5=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F5-G5))</f>
         <v/>
       </c>
       <c r="I5" s="9">
@@ -30701,11 +30701,11 @@
         <v/>
       </c>
       <c r="J5" s="9">
-        <f>IF(OR(B5="",E5=""),"",H5-I5)</f>
+        <f>IF(OR(B5="",E5=""),"",IF(NOT(ISNUMBER(H5)),"ЗАБЛОКИРОВАН",H5-I5))</f>
         <v/>
       </c>
       <c r="K5" s="5">
-        <f>IF(AND(B5="",C5="",D5=""),"",IF(B5="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B5)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D5)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B5)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H5)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J5)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B5="",C5="",D5=""),"",IF(B5="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B5)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D5)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B5)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H5)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J5)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L5" s="5">
@@ -30742,7 +30742,7 @@
         <v/>
       </c>
       <c r="H6" s="9">
-        <f>IF(OR(B6="",E6=""),"",F6-G6)</f>
+        <f>IF(OR(B6="",E6=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F6-G6))</f>
         <v/>
       </c>
       <c r="I6" s="9">
@@ -30750,11 +30750,11 @@
         <v/>
       </c>
       <c r="J6" s="9">
-        <f>IF(OR(B6="",E6=""),"",H6-I6)</f>
+        <f>IF(OR(B6="",E6=""),"",IF(NOT(ISNUMBER(H6)),"ЗАБЛОКИРОВАН",H6-I6))</f>
         <v/>
       </c>
       <c r="K6" s="5">
-        <f>IF(AND(B6="",C6="",D6=""),"",IF(B6="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B6)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D6)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B6)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H6)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J6)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B6="",C6="",D6=""),"",IF(B6="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B6)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D6)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B6)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H6)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J6)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L6" s="5">
@@ -30791,7 +30791,7 @@
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>IF(OR(B7="",E7=""),"",F7-G7)</f>
+        <f>IF(OR(B7="",E7=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F7-G7))</f>
         <v/>
       </c>
       <c r="I7" s="9">
@@ -30799,11 +30799,11 @@
         <v/>
       </c>
       <c r="J7" s="9">
-        <f>IF(OR(B7="",E7=""),"",H7-I7)</f>
+        <f>IF(OR(B7="",E7=""),"",IF(NOT(ISNUMBER(H7)),"ЗАБЛОКИРОВАН",H7-I7))</f>
         <v/>
       </c>
       <c r="K7" s="5">
-        <f>IF(AND(B7="",C7="",D7=""),"",IF(B7="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B7)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D7)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B7)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H7)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J7)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B7="",C7="",D7=""),"",IF(B7="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B7)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D7)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B7)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H7)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J7)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L7" s="5">
@@ -30840,7 +30840,7 @@
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>IF(OR(B8="",E8=""),"",F8-G8)</f>
+        <f>IF(OR(B8="",E8=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F8-G8))</f>
         <v/>
       </c>
       <c r="I8" s="9">
@@ -30848,11 +30848,11 @@
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>IF(OR(B8="",E8=""),"",H8-I8)</f>
+        <f>IF(OR(B8="",E8=""),"",IF(NOT(ISNUMBER(H8)),"ЗАБЛОКИРОВАН",H8-I8))</f>
         <v/>
       </c>
       <c r="K8" s="5">
-        <f>IF(AND(B8="",C8="",D8=""),"",IF(B8="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B8)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D8)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B8)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H8)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J8)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B8="",C8="",D8=""),"",IF(B8="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B8)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D8)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B8)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H8)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J8)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L8" s="5">
@@ -30889,7 +30889,7 @@
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>IF(OR(B9="",E9=""),"",F9-G9)</f>
+        <f>IF(OR(B9="",E9=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F9-G9))</f>
         <v/>
       </c>
       <c r="I9" s="9">
@@ -30897,11 +30897,11 @@
         <v/>
       </c>
       <c r="J9" s="9">
-        <f>IF(OR(B9="",E9=""),"",H9-I9)</f>
+        <f>IF(OR(B9="",E9=""),"",IF(NOT(ISNUMBER(H9)),"ЗАБЛОКИРОВАН",H9-I9))</f>
         <v/>
       </c>
       <c r="K9" s="5">
-        <f>IF(AND(B9="",C9="",D9=""),"",IF(B9="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B9)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D9)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B9)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H9)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J9)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B9="",C9="",D9=""),"",IF(B9="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B9)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D9)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B9)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H9)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J9)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L9" s="5">
@@ -30929,7 +30929,7 @@
         <v/>
       </c>
       <c r="H10" s="9">
-        <f>IF(OR(B10="",E10=""),"",F10-G10)</f>
+        <f>IF(OR(B10="",E10=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F10-G10))</f>
         <v/>
       </c>
       <c r="I10" s="9">
@@ -30937,11 +30937,11 @@
         <v/>
       </c>
       <c r="J10" s="9">
-        <f>IF(OR(B10="",E10=""),"",H10-I10)</f>
+        <f>IF(OR(B10="",E10=""),"",IF(NOT(ISNUMBER(H10)),"ЗАБЛОКИРОВАН",H10-I10))</f>
         <v/>
       </c>
       <c r="K10" s="5">
-        <f>IF(AND(B10="",C10="",D10=""),"",IF(B10="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B10)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D10)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B10)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H10)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J10)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B10="",C10="",D10=""),"",IF(B10="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B10)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D10)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B10)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H10)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J10)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L10" s="5">
@@ -30969,7 +30969,7 @@
         <v/>
       </c>
       <c r="H11" s="9">
-        <f>IF(OR(B11="",E11=""),"",F11-G11)</f>
+        <f>IF(OR(B11="",E11=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F11-G11))</f>
         <v/>
       </c>
       <c r="I11" s="9">
@@ -30977,11 +30977,11 @@
         <v/>
       </c>
       <c r="J11" s="9">
-        <f>IF(OR(B11="",E11=""),"",H11-I11)</f>
+        <f>IF(OR(B11="",E11=""),"",IF(NOT(ISNUMBER(H11)),"ЗАБЛОКИРОВАН",H11-I11))</f>
         <v/>
       </c>
       <c r="K11" s="5">
-        <f>IF(AND(B11="",C11="",D11=""),"",IF(B11="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B11)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D11)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B11)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H11)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J11)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B11="",C11="",D11=""),"",IF(B11="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B11)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D11)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B11)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H11)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J11)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L11" s="5">
@@ -31009,7 +31009,7 @@
         <v/>
       </c>
       <c r="H12" s="9">
-        <f>IF(OR(B12="",E12=""),"",F12-G12)</f>
+        <f>IF(OR(B12="",E12=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F12-G12))</f>
         <v/>
       </c>
       <c r="I12" s="9">
@@ -31017,11 +31017,11 @@
         <v/>
       </c>
       <c r="J12" s="9">
-        <f>IF(OR(B12="",E12=""),"",H12-I12)</f>
+        <f>IF(OR(B12="",E12=""),"",IF(NOT(ISNUMBER(H12)),"ЗАБЛОКИРОВАН",H12-I12))</f>
         <v/>
       </c>
       <c r="K12" s="5">
-        <f>IF(AND(B12="",C12="",D12=""),"",IF(B12="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B12)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D12)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B12)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H12)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J12)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B12="",C12="",D12=""),"",IF(B12="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B12)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D12)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B12)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H12)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J12)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L12" s="5">
@@ -31049,7 +31049,7 @@
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>IF(OR(B13="",E13=""),"",F13-G13)</f>
+        <f>IF(OR(B13="",E13=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F13-G13))</f>
         <v/>
       </c>
       <c r="I13" s="9">
@@ -31057,11 +31057,11 @@
         <v/>
       </c>
       <c r="J13" s="9">
-        <f>IF(OR(B13="",E13=""),"",H13-I13)</f>
+        <f>IF(OR(B13="",E13=""),"",IF(NOT(ISNUMBER(H13)),"ЗАБЛОКИРОВАН",H13-I13))</f>
         <v/>
       </c>
       <c r="K13" s="5">
-        <f>IF(AND(B13="",C13="",D13=""),"",IF(B13="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B13)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D13)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B13)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H13)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J13)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B13="",C13="",D13=""),"",IF(B13="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B13)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D13)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B13)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H13)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J13)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L13" s="5">
@@ -31089,7 +31089,7 @@
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>IF(OR(B14="",E14=""),"",F14-G14)</f>
+        <f>IF(OR(B14="",E14=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F14-G14))</f>
         <v/>
       </c>
       <c r="I14" s="9">
@@ -31097,11 +31097,11 @@
         <v/>
       </c>
       <c r="J14" s="9">
-        <f>IF(OR(B14="",E14=""),"",H14-I14)</f>
+        <f>IF(OR(B14="",E14=""),"",IF(NOT(ISNUMBER(H14)),"ЗАБЛОКИРОВАН",H14-I14))</f>
         <v/>
       </c>
       <c r="K14" s="5">
-        <f>IF(AND(B14="",C14="",D14=""),"",IF(B14="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B14)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D14)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B14)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H14)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J14)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B14="",C14="",D14=""),"",IF(B14="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B14)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D14)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B14)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H14)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J14)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L14" s="5">
@@ -31129,7 +31129,7 @@
         <v/>
       </c>
       <c r="H15" s="9">
-        <f>IF(OR(B15="",E15=""),"",F15-G15)</f>
+        <f>IF(OR(B15="",E15=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F15-G15))</f>
         <v/>
       </c>
       <c r="I15" s="9">
@@ -31137,11 +31137,11 @@
         <v/>
       </c>
       <c r="J15" s="9">
-        <f>IF(OR(B15="",E15=""),"",H15-I15)</f>
+        <f>IF(OR(B15="",E15=""),"",IF(NOT(ISNUMBER(H15)),"ЗАБЛОКИРОВАН",H15-I15))</f>
         <v/>
       </c>
       <c r="K15" s="5">
-        <f>IF(AND(B15="",C15="",D15=""),"",IF(B15="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B15)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D15)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B15)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H15)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J15)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B15="",C15="",D15=""),"",IF(B15="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B15)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D15)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B15)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H15)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J15)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L15" s="5">
@@ -31169,7 +31169,7 @@
         <v/>
       </c>
       <c r="H16" s="9">
-        <f>IF(OR(B16="",E16=""),"",F16-G16)</f>
+        <f>IF(OR(B16="",E16=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F16-G16))</f>
         <v/>
       </c>
       <c r="I16" s="9">
@@ -31177,11 +31177,11 @@
         <v/>
       </c>
       <c r="J16" s="9">
-        <f>IF(OR(B16="",E16=""),"",H16-I16)</f>
+        <f>IF(OR(B16="",E16=""),"",IF(NOT(ISNUMBER(H16)),"ЗАБЛОКИРОВАН",H16-I16))</f>
         <v/>
       </c>
       <c r="K16" s="5">
-        <f>IF(AND(B16="",C16="",D16=""),"",IF(B16="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B16)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D16)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B16)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H16)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J16)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B16="",C16="",D16=""),"",IF(B16="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B16)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D16)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B16)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H16)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J16)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L16" s="5">
@@ -31209,7 +31209,7 @@
         <v/>
       </c>
       <c r="H17" s="9">
-        <f>IF(OR(B17="",E17=""),"",F17-G17)</f>
+        <f>IF(OR(B17="",E17=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F17-G17))</f>
         <v/>
       </c>
       <c r="I17" s="9">
@@ -31217,11 +31217,11 @@
         <v/>
       </c>
       <c r="J17" s="9">
-        <f>IF(OR(B17="",E17=""),"",H17-I17)</f>
+        <f>IF(OR(B17="",E17=""),"",IF(NOT(ISNUMBER(H17)),"ЗАБЛОКИРОВАН",H17-I17))</f>
         <v/>
       </c>
       <c r="K17" s="5">
-        <f>IF(AND(B17="",C17="",D17=""),"",IF(B17="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B17)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D17)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B17)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H17)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J17)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B17="",C17="",D17=""),"",IF(B17="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B17)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D17)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B17)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H17)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J17)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L17" s="5">
@@ -31249,7 +31249,7 @@
         <v/>
       </c>
       <c r="H18" s="9">
-        <f>IF(OR(B18="",E18=""),"",F18-G18)</f>
+        <f>IF(OR(B18="",E18=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F18-G18))</f>
         <v/>
       </c>
       <c r="I18" s="9">
@@ -31257,11 +31257,11 @@
         <v/>
       </c>
       <c r="J18" s="9">
-        <f>IF(OR(B18="",E18=""),"",H18-I18)</f>
+        <f>IF(OR(B18="",E18=""),"",IF(NOT(ISNUMBER(H18)),"ЗАБЛОКИРОВАН",H18-I18))</f>
         <v/>
       </c>
       <c r="K18" s="5">
-        <f>IF(AND(B18="",C18="",D18=""),"",IF(B18="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B18)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D18)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B18)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H18)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J18)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B18="",C18="",D18=""),"",IF(B18="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B18)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D18)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B18)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H18)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J18)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L18" s="5">
@@ -31289,7 +31289,7 @@
         <v/>
       </c>
       <c r="H19" s="9">
-        <f>IF(OR(B19="",E19=""),"",F19-G19)</f>
+        <f>IF(OR(B19="",E19=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F19-G19))</f>
         <v/>
       </c>
       <c r="I19" s="9">
@@ -31297,11 +31297,11 @@
         <v/>
       </c>
       <c r="J19" s="9">
-        <f>IF(OR(B19="",E19=""),"",H19-I19)</f>
+        <f>IF(OR(B19="",E19=""),"",IF(NOT(ISNUMBER(H19)),"ЗАБЛОКИРОВАН",H19-I19))</f>
         <v/>
       </c>
       <c r="K19" s="5">
-        <f>IF(AND(B19="",C19="",D19=""),"",IF(B19="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B19)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D19)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B19)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H19)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J19)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B19="",C19="",D19=""),"",IF(B19="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B19)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D19)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B19)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H19)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J19)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L19" s="5">
@@ -31329,7 +31329,7 @@
         <v/>
       </c>
       <c r="H20" s="9">
-        <f>IF(OR(B20="",E20=""),"",F20-G20)</f>
+        <f>IF(OR(B20="",E20=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F20-G20))</f>
         <v/>
       </c>
       <c r="I20" s="9">
@@ -31337,11 +31337,11 @@
         <v/>
       </c>
       <c r="J20" s="9">
-        <f>IF(OR(B20="",E20=""),"",H20-I20)</f>
+        <f>IF(OR(B20="",E20=""),"",IF(NOT(ISNUMBER(H20)),"ЗАБЛОКИРОВАН",H20-I20))</f>
         <v/>
       </c>
       <c r="K20" s="5">
-        <f>IF(AND(B20="",C20="",D20=""),"",IF(B20="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B20)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D20)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B20)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H20)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J20)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B20="",C20="",D20=""),"",IF(B20="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B20)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D20)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B20)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H20)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J20)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L20" s="5">
@@ -31369,7 +31369,7 @@
         <v/>
       </c>
       <c r="H21" s="9">
-        <f>IF(OR(B21="",E21=""),"",F21-G21)</f>
+        <f>IF(OR(B21="",E21=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F21-G21))</f>
         <v/>
       </c>
       <c r="I21" s="9">
@@ -31377,11 +31377,11 @@
         <v/>
       </c>
       <c r="J21" s="9">
-        <f>IF(OR(B21="",E21=""),"",H21-I21)</f>
+        <f>IF(OR(B21="",E21=""),"",IF(NOT(ISNUMBER(H21)),"ЗАБЛОКИРОВАН",H21-I21))</f>
         <v/>
       </c>
       <c r="K21" s="5">
-        <f>IF(AND(B21="",C21="",D21=""),"",IF(B21="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B21)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D21)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B21)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H21)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J21)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B21="",C21="",D21=""),"",IF(B21="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B21)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D21)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B21)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H21)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J21)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L21" s="5">
@@ -31409,7 +31409,7 @@
         <v/>
       </c>
       <c r="H22" s="9">
-        <f>IF(OR(B22="",E22=""),"",F22-G22)</f>
+        <f>IF(OR(B22="",E22=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F22-G22))</f>
         <v/>
       </c>
       <c r="I22" s="9">
@@ -31417,11 +31417,11 @@
         <v/>
       </c>
       <c r="J22" s="9">
-        <f>IF(OR(B22="",E22=""),"",H22-I22)</f>
+        <f>IF(OR(B22="",E22=""),"",IF(NOT(ISNUMBER(H22)),"ЗАБЛОКИРОВАН",H22-I22))</f>
         <v/>
       </c>
       <c r="K22" s="5">
-        <f>IF(AND(B22="",C22="",D22=""),"",IF(B22="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B22)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D22)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B22)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H22)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J22)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B22="",C22="",D22=""),"",IF(B22="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B22)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D22)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B22)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H22)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J22)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L22" s="5">
@@ -31449,7 +31449,7 @@
         <v/>
       </c>
       <c r="H23" s="9">
-        <f>IF(OR(B23="",E23=""),"",F23-G23)</f>
+        <f>IF(OR(B23="",E23=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F23-G23))</f>
         <v/>
       </c>
       <c r="I23" s="9">
@@ -31457,11 +31457,11 @@
         <v/>
       </c>
       <c r="J23" s="9">
-        <f>IF(OR(B23="",E23=""),"",H23-I23)</f>
+        <f>IF(OR(B23="",E23=""),"",IF(NOT(ISNUMBER(H23)),"ЗАБЛОКИРОВАН",H23-I23))</f>
         <v/>
       </c>
       <c r="K23" s="5">
-        <f>IF(AND(B23="",C23="",D23=""),"",IF(B23="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B23)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D23)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B23)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H23)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J23)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B23="",C23="",D23=""),"",IF(B23="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B23)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D23)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B23)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H23)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J23)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L23" s="5">
@@ -31489,7 +31489,7 @@
         <v/>
       </c>
       <c r="H24" s="9">
-        <f>IF(OR(B24="",E24=""),"",F24-G24)</f>
+        <f>IF(OR(B24="",E24=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F24-G24))</f>
         <v/>
       </c>
       <c r="I24" s="9">
@@ -31497,11 +31497,11 @@
         <v/>
       </c>
       <c r="J24" s="9">
-        <f>IF(OR(B24="",E24=""),"",H24-I24)</f>
+        <f>IF(OR(B24="",E24=""),"",IF(NOT(ISNUMBER(H24)),"ЗАБЛОКИРОВАН",H24-I24))</f>
         <v/>
       </c>
       <c r="K24" s="5">
-        <f>IF(AND(B24="",C24="",D24=""),"",IF(B24="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B24)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D24)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B24)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H24)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J24)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B24="",C24="",D24=""),"",IF(B24="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B24)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D24)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B24)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H24)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J24)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L24" s="5">
@@ -31529,7 +31529,7 @@
         <v/>
       </c>
       <c r="H25" s="9">
-        <f>IF(OR(B25="",E25=""),"",F25-G25)</f>
+        <f>IF(OR(B25="",E25=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F25-G25))</f>
         <v/>
       </c>
       <c r="I25" s="9">
@@ -31537,11 +31537,11 @@
         <v/>
       </c>
       <c r="J25" s="9">
-        <f>IF(OR(B25="",E25=""),"",H25-I25)</f>
+        <f>IF(OR(B25="",E25=""),"",IF(NOT(ISNUMBER(H25)),"ЗАБЛОКИРОВАН",H25-I25))</f>
         <v/>
       </c>
       <c r="K25" s="5">
-        <f>IF(AND(B25="",C25="",D25=""),"",IF(B25="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B25)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D25)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B25)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H25)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J25)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B25="",C25="",D25=""),"",IF(B25="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B25)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D25)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B25)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H25)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J25)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L25" s="5">
@@ -31569,7 +31569,7 @@
         <v/>
       </c>
       <c r="H26" s="9">
-        <f>IF(OR(B26="",E26=""),"",F26-G26)</f>
+        <f>IF(OR(B26="",E26=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F26-G26))</f>
         <v/>
       </c>
       <c r="I26" s="9">
@@ -31577,11 +31577,11 @@
         <v/>
       </c>
       <c r="J26" s="9">
-        <f>IF(OR(B26="",E26=""),"",H26-I26)</f>
+        <f>IF(OR(B26="",E26=""),"",IF(NOT(ISNUMBER(H26)),"ЗАБЛОКИРОВАН",H26-I26))</f>
         <v/>
       </c>
       <c r="K26" s="5">
-        <f>IF(AND(B26="",C26="",D26=""),"",IF(B26="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B26)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D26)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B26)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H26)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J26)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B26="",C26="",D26=""),"",IF(B26="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B26)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D26)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B26)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H26)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J26)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L26" s="5">
@@ -31609,7 +31609,7 @@
         <v/>
       </c>
       <c r="H27" s="9">
-        <f>IF(OR(B27="",E27=""),"",F27-G27)</f>
+        <f>IF(OR(B27="",E27=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F27-G27))</f>
         <v/>
       </c>
       <c r="I27" s="9">
@@ -31617,11 +31617,11 @@
         <v/>
       </c>
       <c r="J27" s="9">
-        <f>IF(OR(B27="",E27=""),"",H27-I27)</f>
+        <f>IF(OR(B27="",E27=""),"",IF(NOT(ISNUMBER(H27)),"ЗАБЛОКИРОВАН",H27-I27))</f>
         <v/>
       </c>
       <c r="K27" s="5">
-        <f>IF(AND(B27="",C27="",D27=""),"",IF(B27="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B27)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D27)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B27)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H27)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J27)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B27="",C27="",D27=""),"",IF(B27="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B27)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D27)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B27)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H27)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J27)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L27" s="5">
@@ -31649,7 +31649,7 @@
         <v/>
       </c>
       <c r="H28" s="9">
-        <f>IF(OR(B28="",E28=""),"",F28-G28)</f>
+        <f>IF(OR(B28="",E28=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F28-G28))</f>
         <v/>
       </c>
       <c r="I28" s="9">
@@ -31657,11 +31657,11 @@
         <v/>
       </c>
       <c r="J28" s="9">
-        <f>IF(OR(B28="",E28=""),"",H28-I28)</f>
+        <f>IF(OR(B28="",E28=""),"",IF(NOT(ISNUMBER(H28)),"ЗАБЛОКИРОВАН",H28-I28))</f>
         <v/>
       </c>
       <c r="K28" s="5">
-        <f>IF(AND(B28="",C28="",D28=""),"",IF(B28="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B28)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D28)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B28)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H28)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J28)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B28="",C28="",D28=""),"",IF(B28="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B28)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D28)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B28)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H28)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J28)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L28" s="5">
@@ -31689,7 +31689,7 @@
         <v/>
       </c>
       <c r="H29" s="9">
-        <f>IF(OR(B29="",E29=""),"",F29-G29)</f>
+        <f>IF(OR(B29="",E29=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F29-G29))</f>
         <v/>
       </c>
       <c r="I29" s="9">
@@ -31697,11 +31697,11 @@
         <v/>
       </c>
       <c r="J29" s="9">
-        <f>IF(OR(B29="",E29=""),"",H29-I29)</f>
+        <f>IF(OR(B29="",E29=""),"",IF(NOT(ISNUMBER(H29)),"ЗАБЛОКИРОВАН",H29-I29))</f>
         <v/>
       </c>
       <c r="K29" s="5">
-        <f>IF(AND(B29="",C29="",D29=""),"",IF(B29="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B29)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D29)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B29)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H29)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J29)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B29="",C29="",D29=""),"",IF(B29="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B29)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D29)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B29)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H29)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J29)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L29" s="5">
@@ -31729,7 +31729,7 @@
         <v/>
       </c>
       <c r="H30" s="9">
-        <f>IF(OR(B30="",E30=""),"",F30-G30)</f>
+        <f>IF(OR(B30="",E30=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F30-G30))</f>
         <v/>
       </c>
       <c r="I30" s="9">
@@ -31737,11 +31737,11 @@
         <v/>
       </c>
       <c r="J30" s="9">
-        <f>IF(OR(B30="",E30=""),"",H30-I30)</f>
+        <f>IF(OR(B30="",E30=""),"",IF(NOT(ISNUMBER(H30)),"ЗАБЛОКИРОВАН",H30-I30))</f>
         <v/>
       </c>
       <c r="K30" s="5">
-        <f>IF(AND(B30="",C30="",D30=""),"",IF(B30="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B30)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D30)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B30)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H30)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J30)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B30="",C30="",D30=""),"",IF(B30="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B30)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D30)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B30)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H30)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J30)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L30" s="5">
@@ -31769,7 +31769,7 @@
         <v/>
       </c>
       <c r="H31" s="9">
-        <f>IF(OR(B31="",E31=""),"",F31-G31)</f>
+        <f>IF(OR(B31="",E31=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F31-G31))</f>
         <v/>
       </c>
       <c r="I31" s="9">
@@ -31777,11 +31777,11 @@
         <v/>
       </c>
       <c r="J31" s="9">
-        <f>IF(OR(B31="",E31=""),"",H31-I31)</f>
+        <f>IF(OR(B31="",E31=""),"",IF(NOT(ISNUMBER(H31)),"ЗАБЛОКИРОВАН",H31-I31))</f>
         <v/>
       </c>
       <c r="K31" s="5">
-        <f>IF(AND(B31="",C31="",D31=""),"",IF(B31="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B31)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D31)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B31)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H31)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J31)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B31="",C31="",D31=""),"",IF(B31="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B31)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D31)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B31)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H31)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J31)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L31" s="5">
@@ -31809,7 +31809,7 @@
         <v/>
       </c>
       <c r="H32" s="9">
-        <f>IF(OR(B32="",E32=""),"",F32-G32)</f>
+        <f>IF(OR(B32="",E32=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F32-G32))</f>
         <v/>
       </c>
       <c r="I32" s="9">
@@ -31817,11 +31817,11 @@
         <v/>
       </c>
       <c r="J32" s="9">
-        <f>IF(OR(B32="",E32=""),"",H32-I32)</f>
+        <f>IF(OR(B32="",E32=""),"",IF(NOT(ISNUMBER(H32)),"ЗАБЛОКИРОВАН",H32-I32))</f>
         <v/>
       </c>
       <c r="K32" s="5">
-        <f>IF(AND(B32="",C32="",D32=""),"",IF(B32="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B32)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D32)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B32)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H32)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J32)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B32="",C32="",D32=""),"",IF(B32="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B32)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D32)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B32)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H32)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J32)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L32" s="5">
@@ -31849,7 +31849,7 @@
         <v/>
       </c>
       <c r="H33" s="9">
-        <f>IF(OR(B33="",E33=""),"",F33-G33)</f>
+        <f>IF(OR(B33="",E33=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F33-G33))</f>
         <v/>
       </c>
       <c r="I33" s="9">
@@ -31857,11 +31857,11 @@
         <v/>
       </c>
       <c r="J33" s="9">
-        <f>IF(OR(B33="",E33=""),"",H33-I33)</f>
+        <f>IF(OR(B33="",E33=""),"",IF(NOT(ISNUMBER(H33)),"ЗАБЛОКИРОВАН",H33-I33))</f>
         <v/>
       </c>
       <c r="K33" s="5">
-        <f>IF(AND(B33="",C33="",D33=""),"",IF(B33="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B33)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D33)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B33)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H33)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J33)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B33="",C33="",D33=""),"",IF(B33="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B33)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D33)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B33)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H33)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J33)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L33" s="5">
@@ -31889,7 +31889,7 @@
         <v/>
       </c>
       <c r="H34" s="9">
-        <f>IF(OR(B34="",E34=""),"",F34-G34)</f>
+        <f>IF(OR(B34="",E34=""),"",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"ЗАБЛОКИРОВАН",F34-G34))</f>
         <v/>
       </c>
       <c r="I34" s="9">
@@ -31897,11 +31897,11 @@
         <v/>
       </c>
       <c r="J34" s="9">
-        <f>IF(OR(B34="",E34=""),"",H34-I34)</f>
+        <f>IF(OR(B34="",E34=""),"",IF(NOT(ISNUMBER(H34)),"ЗАБЛОКИРОВАН",H34-I34))</f>
         <v/>
       </c>
       <c r="K34" s="5">
-        <f>IF(AND(B34="",C34="",D34=""),"",IF(B34="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B34)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D34)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B34)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(N(H34)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J34)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок")))))))</f>
+        <f>IF(AND(B34="",C34="",D34=""),"",IF(B34="","БЛОК: нужен идентификатор акта — по нему распределяются оплаты",IF(COUNTIF($B$5:$B$34,B34)&gt;1,"БЛОК: идентификатор акта повторяется — оплату нельзя отнести однозначно",IF(NOT(ISNUMBER(D34)),"БЛОК: нужен последний день срока оплаты по этому акту",IF(COUNTIF(Взаиморасчёты!$F$5:$F$504,B34)=0,"БЛОК: во «Взаиморасчётах» нет ни одной операции по этому акту",IF(NOT(ISNUMBER(Взаиморасчёты!$M$10)),"БЛОК: реестр «Взаиморасчёты» заблокирован (например, двойной учёт аванса или платёж без акта) — исправьте строки с «БЛОК»: до этого долг по акту не посчитан и в файл 14 не переносится",IF(N(H34)&lt;0,"БЛОК: до первого дня просрочки оплачено и зачтено больше, чем начислено по акту — проверьте распределение",IF(N(J34)&lt;0,"БЛОК: оплаты с первого дня просрочки больше долга на первый день просрочки — проверьте распределение","ок"))))))))</f>
         <v/>
       </c>
       <c r="L34" s="5">

</xml_diff>